<commit_message>
Replace UK30 with UK100
</commit_message>
<xml_diff>
--- a/mosaic_dev/Tickers.xlsx
+++ b/mosaic_dev/Tickers.xlsx
@@ -381,7 +381,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>UK30</t>
+          <t>UK100</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -445,7 +445,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>AZN.L</t>
+          <t>III.L</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -477,7 +477,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>SHEL.L</t>
+          <t>ABDN.L</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>HSBA.L</t>
+          <t>ADM.L</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>ULVR.L</t>
+          <t>AAF.L</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>BP.L</t>
+          <t>ALW.L</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>GSK.L</t>
+          <t>AAL.L</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>RIO.L</t>
+          <t>ANTO.L</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>REL.L</t>
+          <t>ABF.L</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>DGE.L</t>
+          <t>AZN.L</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>BATS.L</t>
+          <t>AUTO.L</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>NG.L</t>
+          <t>AV.L</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>LSEG.L</t>
+          <t>BAB.L</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>BARC.L</t>
+          <t>BA.L</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>LLOY.L</t>
+          <t>BARC.L</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>PRU.L</t>
+          <t>BTRW.L</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>GLEN.L</t>
+          <t>BEZ.L</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>NWG.L</t>
+          <t>BP.L</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>VOD.L</t>
+          <t>BATS.L</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>AAL.L</t>
+          <t>BLND.L</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>STAN.L</t>
+          <t>BT-A.L</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>CPG.L</t>
+          <t>BNZL.L</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>EXPN.L</t>
+          <t>BRBY.L</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>IMB.L</t>
+          <t>CNA.L</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>HLN.L</t>
+          <t>CCEP.L</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>AV.L</t>
+          <t>CCH.L</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>MNG.L</t>
+          <t>CPG.L</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>SMIN.L</t>
+          <t>CCC.L</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>BA.L</t>
+          <t>CTEC.L</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>ENT.L</t>
+          <t>CRDA.L</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>SGE.L</t>
+          <t>DCC.L</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
@@ -1403,6 +1403,11 @@
           <t>REC.MI</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>DGE.L</t>
+        </is>
+      </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
           <t>CON.DE</t>
@@ -1430,6 +1435,11 @@
           <t>SPM.MI</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>DPLM.L</t>
+        </is>
+      </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
           <t>BEI.DE</t>
@@ -1457,6 +1467,11 @@
           <t>SRG.MI</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>EDV.L</t>
+        </is>
+      </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
           <t>IFX.DE</t>
@@ -1484,6 +1499,11 @@
           <t>STLAM.MI</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ENT.L</t>
+        </is>
+      </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
           <t>EOAN.DE</t>
@@ -1511,6 +1531,11 @@
           <t>STMMI.MI</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>EXPN.L</t>
+        </is>
+      </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
           <t>HNR1.DE</t>
@@ -1538,6 +1563,11 @@
           <t>TIT.MI</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>FCIT.L</t>
+        </is>
+      </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
           <t>AIR.DE</t>
@@ -1565,6 +1595,11 @@
           <t>TEN.MI</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FRES.L</t>
+        </is>
+      </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
           <t>SHL.DE</t>
@@ -1592,6 +1627,11 @@
           <t>TRN.MI</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>GAW.L</t>
+        </is>
+      </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
           <t>ENR.DE</t>
@@ -1619,6 +1659,11 @@
           <t>UCG.MI</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>GLEN.L</t>
+        </is>
+      </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
           <t>DTG.DE</t>
@@ -1646,6 +1691,11 @@
           <t>UNI.MI</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>GSK.L</t>
+        </is>
+      </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
           <t>P911.DE</t>
@@ -1668,6 +1718,11 @@
           <t>SIE.DE</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>HLN.L</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
@@ -1685,6 +1740,11 @@
           <t>STLAM.MI</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>HLMA.L</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
@@ -1702,6 +1762,11 @@
           <t>SU.PA</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>HSX.L</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
@@ -1719,6 +1784,11 @@
           <t>SHEL.L</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>HWDN.L</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -1736,6 +1806,11 @@
           <t>TTE.PA</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>HSBA.L</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
@@ -1753,6 +1828,11 @@
           <t>UCG.MI</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ICG.L</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -1770,6 +1850,11 @@
           <t>VOW3.DE</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>IGG.L</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
@@ -1787,6 +1872,11 @@
           <t>VNA.DE</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>IHG.L</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
@@ -1804,6 +1894,11 @@
           <t>VIV.PA</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>IMI.L</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
@@ -1816,6 +1911,11 @@
           <t>CSX</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>IMB.L</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
@@ -1828,6 +1928,11 @@
           <t>ROST</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>INF.L</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
@@ -1840,6 +1945,11 @@
           <t>MNST</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>IAG.L</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
@@ -1852,6 +1962,11 @@
           <t>PAYX</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ITRK.L</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
@@ -1864,6 +1979,11 @@
           <t>AEP</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>INVP.L</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
@@ -1876,6 +1996,11 @@
           <t>PCAR</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>JD.L</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
@@ -1888,6 +2013,11 @@
           <t>KDP</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>BGEO.L</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
@@ -1900,6 +2030,11 @@
           <t>CHTR</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>KGF.L</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
@@ -1912,6 +2047,11 @@
           <t>FAST</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LAND.L</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
@@ -1924,6 +2064,11 @@
           <t>FANG</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LGEN.L</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
@@ -1936,6 +2081,11 @@
           <t>EXC</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LLOY.L</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
@@ -1948,6 +2098,11 @@
           <t>TEAM</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LMP.L</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
@@ -1960,6 +2115,11 @@
           <t>EA</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LSEG.L</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
@@ -1972,6 +2132,11 @@
           <t>XEL</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>MNG.L</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
@@ -1984,6 +2149,11 @@
           <t>ODFL</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>MKS.L</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
@@ -1996,6 +2166,11 @@
           <t>VRSN</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MRO.L</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
@@ -2008,6 +2183,11 @@
           <t>CTSH</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>MTLN.L</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
@@ -2020,6 +2200,11 @@
           <t>KHC</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>NG.L</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
@@ -2032,6 +2217,11 @@
           <t>GEHC</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>NWG.L</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
@@ -2044,6 +2234,11 @@
           <t>IDXX</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>NXT.L</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
@@ -2056,6 +2251,11 @@
           <t>DDOG</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>PSON.L</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
@@ -2068,6 +2268,11 @@
           <t>BIIB</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>PSH.L</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
@@ -2080,6 +2285,11 @@
           <t>DXCM</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>PSN.L</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
@@ -2092,6 +2302,11 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>PCT.L</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
@@ -2104,6 +2319,11 @@
           <t>BKR</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>PRU.L</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
@@ -2116,6 +2336,11 @@
           <t>ZS</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>RKT.L</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
@@ -2128,6 +2353,11 @@
           <t>ANSS</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>REL.L</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="1" t="inlineStr">
@@ -2140,6 +2370,11 @@
           <t>CEG</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>RTO.L</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="1" t="inlineStr">
@@ -2152,6 +2387,11 @@
           <t>DLTR</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>RIO.L</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
@@ -2164,6 +2404,11 @@
           <t>GFS</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>RR.L</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="1" t="inlineStr">
@@ -2176,6 +2421,11 @@
           <t>TTWO</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>SGE.L</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="1" t="inlineStr">
@@ -2188,6 +2438,11 @@
           <t>MDB</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>SBRY.L</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
@@ -2200,6 +2455,11 @@
           <t>ARM</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>SDR.L</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
@@ -2212,6 +2472,11 @@
           <t>DASH</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>SMT.L</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="1" t="inlineStr">
@@ -2224,6 +2489,11 @@
           <t>CCEP</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>SGRO.L</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
@@ -2236,6 +2506,11 @@
           <t>TTD</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>SVT.L</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="1" t="inlineStr">
@@ -2248,6 +2523,11 @@
           <t>MCHP</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>SHEL.L</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
@@ -2260,6 +2540,11 @@
           <t>CDW</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>SMIN.L</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
@@ -2272,6 +2557,11 @@
           <t>AZN</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>SN.L</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="1" t="inlineStr">
@@ -2284,6 +2574,11 @@
           <t>WBD</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>SPX.L</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="1" t="inlineStr">
@@ -2296,6 +2591,11 @@
           <t>SBUX</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>SSE.L</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
@@ -2308,6 +2608,11 @@
           <t>ALGN</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>STAN.L</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="1" t="inlineStr">
@@ -2320,6 +2625,11 @@
           <t>ILMN</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>SDLF.L</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="1" t="inlineStr">
@@ -2332,6 +2642,11 @@
           <t>EBAY</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>STJ.L</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
@@ -2344,6 +2659,11 @@
           <t>SIRI</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>TSCO.L</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="1" t="inlineStr">
@@ -2356,6 +2676,11 @@
           <t>INTC</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>BBOX.L</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="1" t="inlineStr">
@@ -2368,6 +2693,11 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>ULVR.L</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
@@ -2380,6 +2710,11 @@
           <t>ALAB</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>UU.L</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="1" t="inlineStr">
@@ -2392,6 +2727,11 @@
           <t>CRWV</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>VOD.L</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="1" t="inlineStr">
@@ -2404,6 +2744,11 @@
           <t>NBIS</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>WEIR.L</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
@@ -2414,6 +2759,11 @@
       <c r="B102" s="1" t="inlineStr">
         <is>
           <t>RKLB</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>WTB.L</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update weekly Mosaic reports for 2026-07-10
</commit_message>
<xml_diff>
--- a/mosaic_dev/Tickers.xlsx
+++ b/mosaic_dev/Tickers.xlsx
@@ -348,10 +348,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.7109375" customWidth="1" min="1" max="7"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10.28515625" customWidth="1" min="8" max="8"/>
     <col width="8.7109375" customWidth="1" min="9" max="13"/>
     <col width="13" customWidth="1" min="14" max="15"/>
@@ -389,6 +391,11 @@
           <t>Germany40</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Australia50</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -421,6 +428,11 @@
           <t>EWG</t>
         </is>
       </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>EWA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -453,6 +465,11 @@
           <t>SIE.DE</t>
         </is>
       </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>ALL.AX</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -485,6 +502,11 @@
           <t>DTE.DE</t>
         </is>
       </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>AMC.AX</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -517,6 +539,11 @@
           <t>ALV.DE</t>
         </is>
       </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>ANZ.AX</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -549,6 +576,11 @@
           <t>MUV2.DE</t>
         </is>
       </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>ASX.AX</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -581,6 +613,11 @@
           <t>DHL.DE</t>
         </is>
       </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>BHP.AX</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -613,6 +650,11 @@
           <t>BMW.DE</t>
         </is>
       </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>BXB.AX</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -645,6 +687,11 @@
           <t>BAS.DE</t>
         </is>
       </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>CAR.AX</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -677,6 +724,11 @@
           <t>DB1.DE</t>
         </is>
       </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>CBA.AX</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -709,6 +761,11 @@
           <t>CBK.DE</t>
         </is>
       </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>COH.AX</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -741,6 +798,11 @@
           <t>RWE.DE</t>
         </is>
       </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>COL.AX</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -773,6 +835,11 @@
           <t>BAYN.DE</t>
         </is>
       </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>CPU.AX</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -805,6 +872,11 @@
           <t>HEI.DE</t>
         </is>
       </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>CSL.AX</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -837,6 +909,11 @@
           <t>FRE.DE</t>
         </is>
       </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>EVN.AX</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -869,6 +946,11 @@
           <t>VOW3.DE</t>
         </is>
       </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>FMG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -901,6 +983,11 @@
           <t>MRK.DE</t>
         </is>
       </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>FPH.AX</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -933,6 +1020,11 @@
           <t>VNA.DE</t>
         </is>
       </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>GMG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -965,6 +1057,11 @@
           <t>MTX.DE</t>
         </is>
       </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>IAG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -997,6 +1094,11 @@
           <t>HEN3.DE</t>
         </is>
       </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>JBH.AX</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
@@ -1029,6 +1131,11 @@
           <t>FME.DE</t>
         </is>
       </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>JHX.AX</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
@@ -1061,6 +1168,11 @@
           <t>SRT3.DE</t>
         </is>
       </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>LYC.AX</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
@@ -1093,6 +1205,11 @@
           <t>PAH3.DE</t>
         </is>
       </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>MPL.AX</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
@@ -1125,6 +1242,11 @@
           <t>ZAL.DE</t>
         </is>
       </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>MQG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
@@ -1157,6 +1279,11 @@
           <t>ADS.DE</t>
         </is>
       </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>NAB.AX</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -1189,6 +1316,11 @@
           <t>DBK.DE</t>
         </is>
       </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>NEM.AX</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
@@ -1221,6 +1353,11 @@
           <t>RHM.DE</t>
         </is>
       </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>NST.AX</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
@@ -1253,6 +1390,11 @@
           <t>SAP.DE</t>
         </is>
       </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>NWS.AX</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -1285,6 +1427,11 @@
           <t>SY1.DE</t>
         </is>
       </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>ORG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
@@ -1317,6 +1464,11 @@
           <t>BNR.DE</t>
         </is>
       </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>PME.AX</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
@@ -1349,6 +1501,11 @@
           <t>MBG.DE</t>
         </is>
       </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>QAN.AX</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
@@ -1381,6 +1538,11 @@
           <t>QIA.DE</t>
         </is>
       </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>QBE.AX</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
@@ -1413,6 +1575,11 @@
           <t>CON.DE</t>
         </is>
       </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>REA.AX</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
@@ -1445,6 +1612,11 @@
           <t>BEI.DE</t>
         </is>
       </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>RIO.AX</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
@@ -1477,6 +1649,11 @@
           <t>IFX.DE</t>
         </is>
       </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>RMD.AX</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
@@ -1509,6 +1686,11 @@
           <t>EOAN.DE</t>
         </is>
       </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>S32.AX</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
@@ -1541,6 +1723,11 @@
           <t>HNR1.DE</t>
         </is>
       </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>SCG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
@@ -1573,6 +1760,11 @@
           <t>AIR.DE</t>
         </is>
       </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>SGH.AX</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
@@ -1605,6 +1797,11 @@
           <t>SHL.DE</t>
         </is>
       </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>SGP.AX</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
@@ -1637,6 +1834,11 @@
           <t>ENR.DE</t>
         </is>
       </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>SIG.AX</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
@@ -1669,6 +1871,11 @@
           <t>DTG.DE</t>
         </is>
       </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>SOL.AX</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
@@ -1701,6 +1908,11 @@
           <t>P911.DE</t>
         </is>
       </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>STO.AX</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
@@ -1723,6 +1935,11 @@
           <t>HLN.L</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SUN.AX</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
@@ -1745,6 +1962,11 @@
           <t>HLMA.L</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>TCL.AX</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
@@ -1767,6 +1989,11 @@
           <t>HSX.L</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>TLS.AX</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
@@ -1789,6 +2016,11 @@
           <t>HWDN.L</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>WBC.AX</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -1811,6 +2043,11 @@
           <t>HSBA.L</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>WES.AX</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
@@ -1833,6 +2070,11 @@
           <t>ICG.L</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>WDS.AX</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -1855,6 +2097,11 @@
           <t>IGG.L</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>WOW.AX</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
@@ -1877,6 +2124,11 @@
           <t>IHG.L</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>WTC.AX</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
@@ -1899,6 +2151,11 @@
           <t>IMI.L</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>XRO.AX</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
@@ -1914,6 +2171,11 @@
       <c r="E52" t="inlineStr">
         <is>
           <t>IMB.L</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>XYZ.AX</t>
         </is>
       </c>
     </row>

</xml_diff>